<commit_message>
Add explicit Stashaway FX rates for 5/21 deposits; regenerate reports
Deposits sheet now has `FX Rate to base` populated for all cross-currency
new-sleeve seed deposits (Asia ex-Japan, Japan Currency-hedged at 0.7791
matching Global Floating Rate USD; Longevity Stack + AI Power Stack
already at 0.7813). Explicit rates replace the 0.2% midmarket-haircut
fallback so the deposit anchor reflects Stashaway's exact conversion.

Numerical impact small (~$1-2 per sleeve from the haircut approximation
being very close to the actual rate). The larger gap movements are from
one extra trading day (6/1 → 6/2 end_date) of price action.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/holding.xlsx
+++ b/data/holding.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dalva\src\project-hail-mary\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{639C7904-62E6-4364-9805-08629C687371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BAE625C-2D4B-4E50-873C-2198690325BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41850" yWindow="2520" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4980" yWindow="1335" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Holdings" sheetId="1" r:id="rId1"/>
@@ -768,7 +768,7 @@
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -935,12 +935,6 @@
       <name val="Noto Sans"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF666666"/>
-      <name val="Noto Sans"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -970,7 +964,7 @@
     <xf numFmtId="9" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1039,7 +1033,6 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -5721,8 +5714,11 @@
       <c r="E8" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="F8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="24">
         <v>46163</v>
       </c>
@@ -5738,7 +5734,7 @@
       <c r="E9" t="s">
         <v>168</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9">
         <v>0.77910000000000001</v>
       </c>
     </row>
@@ -5758,6 +5754,9 @@
       <c r="E10" t="s">
         <v>168</v>
       </c>
+      <c r="F10">
+        <v>0.77910000000000001</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="24">
@@ -5775,6 +5774,9 @@
       <c r="E11" t="s">
         <v>168</v>
       </c>
+      <c r="F11">
+        <v>0.77910000000000001</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="24">
@@ -5866,7 +5868,7 @@
       <c r="C16" t="s">
         <v>159</v>
       </c>
-      <c r="D16" s="37">
+      <c r="D16" s="36">
         <v>5000</v>
       </c>
       <c r="E16" t="s">

</xml_diff>